<commit_message>
adding in google api for constr companies
</commit_message>
<xml_diff>
--- a/data/leads.xlsx
+++ b/data/leads.xlsx
@@ -16,7 +16,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -55,11 +58,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -459,6 +463,21 @@
           <t>LinkedIn</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Industry</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Date Added</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -491,6 +510,9 @@
           <t>https://linkedin.com/company/mikesplumbing</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -523,6 +545,9 @@
           <t>https://linkedin.com/company/desertairhvac</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -554,6 +579,173 @@
         <is>
           <t>https://linkedin.com/company/phxroofing</t>
         </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Ethan Wells</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Sunset Construction Services</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://sunsetconstructionservices.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>gregperger@gmail.com</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2024-08-28</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Google Maps (sample)</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>46120.81544764517</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Nina Alvarez</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Pinnacle Builders</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>https://pinnaclebuildersaz.com</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>info@pinnaclebuildersaz.com</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>602-555-1234</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Google Maps (sample)</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>46120.81544764536</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Ari Becker</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Ridge Line Builders</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>https://ridgelinebuilders.com</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>dave@ridgelinebuilders.com</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2020-10-20</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Google Maps (sample)</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="n">
+        <v>46120.81544764539</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Ariel Gonzalez</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Phoenix Construction Co</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>https://phoenixconstructionco.com</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>info@phoenixconstructionco.com</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>602-555-1234</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Thumbtack (sample)</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="n">
+        <v>46120.81544764539</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated to be soflo location only and increased number
</commit_message>
<xml_diff>
--- a/data/leads.xlsx
+++ b/data/leads.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -622,7 +622,7 @@
         </is>
       </c>
       <c r="I5" s="2" t="n">
-        <v>46120.81544764517</v>
+        <v>46120.81544765046</v>
       </c>
     </row>
     <row r="6">
@@ -663,7 +663,7 @@
         </is>
       </c>
       <c r="I6" s="2" t="n">
-        <v>46120.81544764536</v>
+        <v>46120.81544765046</v>
       </c>
     </row>
     <row r="7">
@@ -704,7 +704,7 @@
         </is>
       </c>
       <c r="I7" s="2" t="n">
-        <v>46120.81544764539</v>
+        <v>46120.81544765046</v>
       </c>
     </row>
     <row r="8">
@@ -745,7 +745,1866 @@
         </is>
       </c>
       <c r="I8" s="2" t="n">
-        <v>46120.81544764539</v>
+        <v>46120.81544765046</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Carlos Ramirez</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Miami Home Renovations</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>https://mihomesreno.com</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>info@mihomesreno.com</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>602-555-1234</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Google Maps (sample)</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="n">
+        <v>46120.82280933936</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Sofia Lopez</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Palm Beach Contractors</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>https://palmbeachcontractors.com</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>info@palmbeachcontractors.com</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>602-555-1234</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Google Maps (sample)</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="n">
+        <v>46120.82280933944</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Contact 4</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Valley Concrete</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>https://valleyconcrete.com</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>user@domain.com.</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>1618513208426</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Thumbtack (sample)</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="n">
+        <v>46120.82280933946</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Contact 7</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Fort Lauderdale Builders</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>https://fortlauderdalebuilders.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Thumbtack (sample)</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="n">
+        <v>46120.82280933949</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Contact 8</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>South Florida Excavation</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>https://southfloridaexcavation.com</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>info@southfloridaexcavation.com</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>602-555-1234</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Thumbtack (sample)</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="n">
+        <v>46120.8228093395</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Contact 9</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Coastal Construction Co</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>https://coastalconstructionco.com</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>fancybox@3.5.7</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>2021-06-09</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Thumbtack (sample)</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="n">
+        <v>46120.82280933952</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Contact 10</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Tropical Builders</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>https://tropicalbuilders.com</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Thumbtack (sample)</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="n">
+        <v>46120.82280933954</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Contact 11</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Everglades Contractors</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>https://evergladescontractors.com</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>info@evergladescontractors.com</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>602-555-1234</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Thumbtack (sample)</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="n">
+        <v>46120.82280933955</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Contact 12</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Beachside Renovations</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>https://beachsiderenovations.com</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>63101157</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Thumbtack (sample)</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="n">
+        <v>46120.82280933956</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Contact 13</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Key West Construction</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>https://keywestconstruction.com</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>user@domain.com.</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>4211612264</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Thumbtack (sample)</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="n">
+        <v>46120.82280933958</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Contact 14</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Coral Gables Builders</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>https://coralgablesbuilders.com</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>info@coralgablesbuilders.com</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>602-555-1234</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Thumbtack (sample)</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="n">
+        <v>46120.8228093396</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Contact 15</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Brickell Contractors</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>https://brickellcontractors.com</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>info@brickellcontractors.com</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>602-555-1234</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Thumbtack (sample)</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="n">
+        <v>46120.82280933961</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Contact 16</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Wynwood Renovations</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>https://wynwoodrenovations.com</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>info@wynwoodrenovations.com</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>602-555-1234</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Thumbtack (sample)</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="n">
+        <v>46120.82280933962</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Contact 17</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Little Havana Builders</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>https://littlehavanabuilders.com</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>info@littlehavanabuilders.com</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>602-555-1234</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Thumbtack (sample)</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="n">
+        <v>46120.82280933963</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Contact 18</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Doral Construction</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>https://doralconstruction.com</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>info@doralconstruction.com</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>602-555-1234</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Thumbtack (sample)</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="n">
+        <v>46120.82280933964</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Contact 19</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Kendall Contractors</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>https://kendallcontractors.com</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>info@kendallcontractors.com</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>602-555-1234</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Thumbtack (sample)</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="n">
+        <v>46120.82280933965</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Contact 20</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Homestead Builders</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>https://homesteadbuilders.com</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Thumbtack (sample)</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="n">
+        <v>46120.82280933966</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Contact 21</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Cutler Bay Renovations</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>https://cutlerbayrenovations.com</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>info@cutlerbayrenovations.com</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>602-555-1234</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Thumbtack (sample)</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="n">
+        <v>46120.82280933968</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Contact 22</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Pinecrest Construction</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>https://pinecrestconstruction.com</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>info@pinecrestconstruction.com</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>602-555-1234</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Thumbtack (sample)</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="n">
+        <v>46120.82280933969</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Contact 23</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>South Miami Builders</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>https://southmiamibuilders.com</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>+0152-0153</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Thumbtack (sample)</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="n">
+        <v>46120.8228093397</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Contact 24</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Gables Contractors</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>https://gablescontractors.com</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>info@gablescontractors.com</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>602-555-1234</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Thumbtack (sample)</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="n">
+        <v>46120.82280933972</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Contact 25</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Bal Harbour Renovations</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>https://balharbourrenovations.com</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>info@balharbourrenovations.com</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>602-555-1234</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Thumbtack (sample)</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="n">
+        <v>46120.82280933973</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Contact 26</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Surfside Builders</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>https://surfsidebuilders.com</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Thumbtack (sample)</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="n">
+        <v>46120.82280933975</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Contact 27</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Sunny Isles Construction</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>https://sunnyislesconstruction.com</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>info@sunnyislesconstruction.com</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>602-555-1234</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Thumbtack (sample)</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="n">
+        <v>46120.82280933976</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Contact 28</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Aventura Contractors</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>https://aventuracontractors.com</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>info@aventuracontractors.com</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>602-555-1234</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Thumbtack (sample)</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="n">
+        <v>46120.82280933977</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Contact 29</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Hallandale Builders</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>https://hallandalebuilders.com</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>info@hallandalebuilders.com</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>602-555-1234</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Thumbtack (sample)</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="n">
+        <v>46120.82280933978</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Contact 30</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Hollywood Renovations</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>https://hollywoodrenovations.com</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>info@hollywoodrenovations.com</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>602-555-1234</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Thumbtack (sample)</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="n">
+        <v>46120.82280933979</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Contact 31</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Pembroke Pines Construction</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>https://pembrokepinesconstruction.com</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>info@pembrokepinesconstruction.com</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>602-555-1234</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Thumbtack (sample)</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="n">
+        <v>46120.82280933981</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Contact 32</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Miramar Contractors</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>https://miramarcontractors.com</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>info@miramarcontractors.com</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>602-555-1234</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Thumbtack (sample)</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="n">
+        <v>46120.82280933981</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Contact 33</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Davie Builders</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>https://daviebuilders.com</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>+0400-045</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Thumbtack (sample)</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="n">
+        <v>46120.82280933983</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Contact 34</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Cooper City Renovations</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>https://coopercityrenovations.com</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>info@coopercityrenovations.com</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>602-555-1234</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Thumbtack (sample)</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="n">
+        <v>46120.82280933984</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Contact 35</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Weston Construction</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>https://westonconstruction.com</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>info@westonconstruction.com</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>602-555-1234</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Thumbtack (sample)</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="n">
+        <v>46120.82280933985</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Contact 36</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Plantation Contractors</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>https://plantationcontractors.com</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>info@plantationcontractors.com</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>602-555-1234</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Thumbtack (sample)</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="n">
+        <v>46120.82280933987</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Contact 37</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Sunrise Builders</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>https://sunrisebuilders.com</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>info@sunrisebuilders.com</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>602-555-1234</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Thumbtack (sample)</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="n">
+        <v>46120.82280933987</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Contact 38</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Lauderhill Renovations</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>https://lauderhillrenovations.com</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>info@lauderhillrenovations.com</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>602-555-1234</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Thumbtack (sample)</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="n">
+        <v>46120.82280933989</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Contact 39</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Tamarac Construction</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>https://tamaracconstruction.com</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>info@tamaracconstruction.com</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>602-555-1234</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Thumbtack (sample)</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="n">
+        <v>46120.82280933989</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Contact 40</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Coral Springs Contractors</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>https://coralspringscontractors.com</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>info@coralspringscontractors.com</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>602-555-1234</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Thumbtack (sample)</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="n">
+        <v>46120.82280933991</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Contact 41</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Parkland Builders</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>https://parklandbuilders.com</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Thumbtack (sample)</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="n">
+        <v>46120.82280933992</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Contact 42</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Margate Renovations</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>https://margaterenovations.com</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>info@margaterenovations.com</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>602-555-1234</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Thumbtack (sample)</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="n">
+        <v>46120.82280933993</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Contact 43</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Coconut Creek Construction</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>https://coconutcreekconstruction.com</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>info@coconutcreekconstruction.com</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>602-555-1234</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Thumbtack (sample)</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="n">
+        <v>46120.82280933994</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Contact 44</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Deerfield Beach Contractors</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>https://deerfieldbeachcontractors.com</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>info@deerfieldbeachcontractors.com</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>602-555-1234</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Thumbtack (sample)</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I49" s="2" t="n">
+        <v>46120.82280933995</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Contact 45</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Boca Raton Builders</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>https://bocaratonbuilders.com</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Thumbtack (sample)</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="n">
+        <v>46120.82280934009</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Contact 46</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Delray Beach Renovations</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>https://delraybeachrenovations.com</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr"/>
+      <c r="E51" t="inlineStr"/>
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Thumbtack (sample)</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I51" s="2" t="n">
+        <v>46120.8228093401</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Contact 47</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Boynton Beach Construction</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>https://boyntonbeachconstruction.com</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>info@boyntonbeachconstruction.com</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>602-555-1234</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr"/>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Thumbtack (sample)</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="n">
+        <v>46120.82280934011</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Contact 48</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Lake Worth Contractors</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>https://lakeworthcontractors.com</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>info@lakeworthcontractors.com</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>602-555-1234</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr"/>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Thumbtack (sample)</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="n">
+        <v>46120.82280934013</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Contact 49</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>West Palm Beach Builders</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>https://westpalmbeachbuilders.com</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>info@westpalmbeachbuilders.com</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>602-555-1234</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Thumbtack (sample)</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="n">
+        <v>46120.82280934014</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Contact 50</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Palm Beach Gardens Renovations</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>https://palmbeachgardensrenovations.com</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>info@palmbeachgardensrenovations.com</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>602-555-1234</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Thumbtack (sample)</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="n">
+        <v>46120.82280934015</v>
       </c>
     </row>
   </sheetData>

</xml_diff>